<commit_message>
Enhance README and code to support security role assignments in DMF import. Update input structure to include security roles and organization assignments. Modify OData import process to handle new security entities and improve preflight checks. Update CLI prompts and add new command-line options for security role management. Update example input file to reflect changes.
</commit_message>
<xml_diff>
--- a/input/users-example.xlsx
+++ b/input/users-example.xlsx
@@ -1,34 +1,127 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hsdyn-my.sharepoint.com/personal/ilopezcoll_hsdyn_com/Documents/001_Customers/CSC/System Users/input/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D5B796C38444A540CFF050DF18757517F6BA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C0BCD15-101F-4AAE-83F5-43121FD9BE9B}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28035" windowHeight="17910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Users" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+  <si>
+    <t>UserId</t>
+  </si>
+  <si>
+    <t>Alias</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>SecurityRoles</t>
+  </si>
+  <si>
+    <t>SecurityLegalEntityIds</t>
+  </si>
+  <si>
+    <t>SecurityLegalEntities</t>
+  </si>
+  <si>
+    <t>DemoAcct</t>
+  </si>
+  <si>
+    <t>demo.acct@example.com</t>
+  </si>
+  <si>
+    <t>Alex</t>
+  </si>
+  <si>
+    <t>Accountant</t>
+  </si>
+  <si>
+    <t>Accountant, Accounting Manager</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>OPERATIONALLE</t>
+  </si>
+  <si>
+    <t>DemoBasic</t>
+  </si>
+  <si>
+    <t>demo.basic@example.com</t>
+  </si>
+  <si>
+    <t>Blake</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>DemoRoleOnly</t>
+  </si>
+  <si>
+    <t>demo.roleonly@example.com</t>
+  </si>
+  <si>
+    <t>Casey</t>
+  </si>
+  <si>
+    <t>RoleOnly</t>
+  </si>
+  <si>
+    <t>System user</t>
+  </si>
+  <si>
+    <t>DemoMultiLE</t>
+  </si>
+  <si>
+    <t>demo.multile@example.com</t>
+  </si>
+  <si>
+    <t>Dana</t>
+  </si>
+  <si>
+    <t>MultiLE</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +140,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,69 +442,141 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>UserId</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Alias</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>FirstName</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>LastName</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>JDOE</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>jdoe</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>jane.doe@example.com</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Jane</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Doe</t>
-        </is>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{50a58a55-8d55-4c7b-aa85-1ae890a4cc64}" enabled="1" method="Standard" siteId="{e85feadf-11e7-47bb-a160-43b98dcc96f1}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>